<commit_message>
feat: Implement all-or-nothing transaction for Excel imports to ensure data consistency by rolling back the entire operation if any errors are found.
</commit_message>
<xml_diff>
--- a/Backend/test_migration_files/testing_penerimaan_excel.xlsx
+++ b/Backend/test_migration_files/testing_penerimaan_excel.xlsx
@@ -67,18 +67,21 @@
     <t>Bank Mandiri</t>
   </si>
   <si>
+    <t>Zakat Fitrah</t>
+  </si>
+  <si>
+    <t>Individu</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>12.5</t>
+  </si>
+  <si>
     <t>Zakat</t>
   </si>
   <si>
-    <t>Individu</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>12.5</t>
-  </si>
-  <si>
     <t>02 Januari 2026</t>
   </si>
   <si>
@@ -88,7 +91,7 @@
     <t>BSI Zakat</t>
   </si>
   <si>
-    <t>Zakat Perdagangan</t>
+    <t>Zakat Maal</t>
   </si>
   <si>
     <t>Entitas</t>
@@ -107,9 +110,6 @@
   </si>
   <si>
     <t>Kantor Digital</t>
-  </si>
-  <si>
-    <t>Zakat Emas</t>
   </si>
   <si>
     <t>04 Februari 2026</t>
@@ -664,33 +664,33 @@
         <v>20</v>
       </c>
       <c r="M2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
         <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I3">
         <v>5000000</v>
@@ -705,27 +705,27 @@
         <v>20</v>
       </c>
       <c r="M3" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
         <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
         <v>19</v>
@@ -746,7 +746,7 @@
         <v>20</v>
       </c>
       <c r="M4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -754,7 +754,7 @@
         <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
         <v>34</v>
@@ -766,7 +766,7 @@
         <v>35</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="G5" t="s">
         <v>19</v>
@@ -787,7 +787,7 @@
         <v>20</v>
       </c>
       <c r="M5" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -851,7 +851,7 @@
         <v>47</v>
       </c>
       <c r="G7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H7" t="s">
         <v>48</v>
@@ -924,13 +924,13 @@
         <v>56</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="G9" t="s">
         <v>19</v>
@@ -951,7 +951,7 @@
         <v>20</v>
       </c>
       <c r="M9" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -992,7 +992,7 @@
         <v>20</v>
       </c>
       <c r="M10" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -1015,7 +1015,7 @@
         <v>63</v>
       </c>
       <c r="G11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H11" t="s">
         <v>64</v>
@@ -1038,6 +1038,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>